<commit_message>
Import B4 sales Oct 2026 from Parn's Daily Sales Record photos (approved by Parn)
18 days, revenue 43100 before ice (--undated=18); ice in Expenses. Sheets marked B-5/blank booked as B4 per Parn. safe_import_sales.js now accepts B4.
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B4_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B4_2026.xlsx
@@ -134,10 +134,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -169,10 +169,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1520,7 +1520,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF3"/>
+  <dimension ref="A1:AF21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1625,9 +1625,807 @@
         <v>Source Note</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C4">
+        <v>3780</v>
+      </c>
+      <c r="D4">
+        <v>1947</v>
+      </c>
+      <c r="E4">
+        <v>60</v>
+      </c>
+      <c r="G4">
+        <v>1833</v>
+      </c>
+      <c r="H4">
+        <v>8</v>
+      </c>
+      <c r="J4">
+        <v>13</v>
+      </c>
+      <c r="K4">
+        <v>4</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
+      <c r="O4">
+        <v>5</v>
+      </c>
+      <c r="P4">
+        <v>2</v>
+      </c>
+      <c r="Q4">
+        <v>46</v>
+      </c>
+      <c r="AF4" t="str">
+        <v>Parn photo 01M59J90GR140C7NWESP7HBDJE.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 10, Pomegranate 2 | CHECK: branch written "B-5"</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C5">
+        <v>4269</v>
+      </c>
+      <c r="D5">
+        <v>2970</v>
+      </c>
+      <c r="E5">
+        <v>60</v>
+      </c>
+      <c r="G5">
+        <v>1299</v>
+      </c>
+      <c r="H5">
+        <v>11</v>
+      </c>
+      <c r="J5">
+        <v>14</v>
+      </c>
+      <c r="K5">
+        <v>6</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
+      <c r="O5">
+        <v>3</v>
+      </c>
+      <c r="P5">
+        <v>2</v>
+      </c>
+      <c r="Q5">
+        <v>49</v>
+      </c>
+      <c r="AF5" t="str">
+        <v>Parn photo 01M59J91CQJHZ1H6GQWYSH15T0.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Pomegranate 11 | CHECK: branch written "blank"</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>03/10/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C6">
+        <v>5126</v>
+      </c>
+      <c r="D6">
+        <v>2623</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>2503</v>
+      </c>
+      <c r="H6">
+        <v>14</v>
+      </c>
+      <c r="J6">
+        <v>9</v>
+      </c>
+      <c r="K6">
+        <v>4</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+      <c r="O6">
+        <v>2</v>
+      </c>
+      <c r="P6">
+        <v>4</v>
+      </c>
+      <c r="Q6">
+        <v>56</v>
+      </c>
+      <c r="AF6" t="str">
+        <v>Parn photo 01M59J91CE83KN64KME60GJ66C.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 10, Grape 4, Pomegranate 5 | CHECK: branch written "B-5"</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>04/10/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C7">
+        <v>5016</v>
+      </c>
+      <c r="D7">
+        <v>2691</v>
+      </c>
+      <c r="E7">
+        <v>60</v>
+      </c>
+      <c r="G7">
+        <v>2325</v>
+      </c>
+      <c r="H7">
+        <v>7</v>
+      </c>
+      <c r="J7">
+        <v>11</v>
+      </c>
+      <c r="K7">
+        <v>4</v>
+      </c>
+      <c r="M7">
+        <v>4</v>
+      </c>
+      <c r="O7">
+        <v>3</v>
+      </c>
+      <c r="P7">
+        <v>3</v>
+      </c>
+      <c r="Q7">
+        <v>51</v>
+      </c>
+      <c r="AF7" t="str">
+        <v>Parn photo 01M59J9S2F8Z1WNM683T3F3ZER.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 9, Grape 4, Pomegranate 5, Mangosteen no ice 1 | CHECK: cash items 2511 vs written 2691 (+180); branch written "B-5"</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>05/10/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C8">
+        <v>2841</v>
+      </c>
+      <c r="D8">
+        <v>1705</v>
+      </c>
+      <c r="E8">
+        <v>60</v>
+      </c>
+      <c r="G8">
+        <v>1136</v>
+      </c>
+      <c r="H8">
+        <v>4</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>6</v>
+      </c>
+      <c r="K8">
+        <v>2</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
+      </c>
+      <c r="O8">
+        <v>2</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>30</v>
+      </c>
+      <c r="AF8" t="str">
+        <v>Parn photo 01M59J91AM9M9BMFPWVR3PJFEJ.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 8, Grape 2, Pomegranate 3 | CHECK: branch written "B-5"</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>06/10/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C9">
+        <v>1308</v>
+      </c>
+      <c r="D9">
+        <v>869</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>439</v>
+      </c>
+      <c r="H9">
+        <v>2</v>
+      </c>
+      <c r="J9">
+        <v>2</v>
+      </c>
+      <c r="K9">
+        <v>5</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>1</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>14</v>
+      </c>
+      <c r="AF9" t="str">
+        <v>Parn photo 01M59J9K44G95R8NMDKVV135ZR.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 2, Grape 1, Pomegranate 1 | CHECK: branch written "B-5"</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>07/10/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C10">
+        <v>1378</v>
+      </c>
+      <c r="D10">
+        <v>380</v>
+      </c>
+      <c r="E10">
+        <v>60</v>
+      </c>
+      <c r="G10">
+        <v>998</v>
+      </c>
+      <c r="H10">
+        <v>4</v>
+      </c>
+      <c r="J10">
+        <v>10</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>1</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>19</v>
+      </c>
+      <c r="AF10" t="str">
+        <v>Parn photo 01M59J9NN1659SB4KXXHTQHHYN.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 2, Pomegranate 1 | CHECK: branch written "B-04"</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>08/10/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C11">
+        <v>1963</v>
+      </c>
+      <c r="D11">
+        <v>1086</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>877</v>
+      </c>
+      <c r="H11">
+        <v>2</v>
+      </c>
+      <c r="J11">
+        <v>2</v>
+      </c>
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="M11">
+        <v>5</v>
+      </c>
+      <c r="O11">
+        <v>3</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>23</v>
+      </c>
+      <c r="AF11" t="str">
+        <v>Parn photo 01M59J91C84W60ZV60XAC5R6V3.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 4, Pomegranate 2, Grape 4 | CHECK: cash items 1089 vs booked 1086 (-3); branch written "B-04"; ice 60 written then crossed out; Parn 19/10/2026: book written grand total 1963 (not 1966); 3 taken off cash (1089 -&gt; 1086), QR 877 unchanged</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C12">
+        <v>1246</v>
+      </c>
+      <c r="D12">
+        <v>886</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>360</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>4</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>2</v>
+      </c>
+      <c r="O12">
+        <v>3</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>15</v>
+      </c>
+      <c r="AF12" t="str">
+        <v>Parn photo 01M59J91D2ZT3CV2DWW9GJGHC0.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 4, Pomegranate 1, Grape 1 | CHECK: no grand total written; cash 886 + QR 360 = 1246; branch written "B-04"</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>10/10/2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C13">
+        <v>2562</v>
+      </c>
+      <c r="D13">
+        <v>1713</v>
+      </c>
+      <c r="E13">
+        <v>60</v>
+      </c>
+      <c r="G13">
+        <v>849</v>
+      </c>
+      <c r="H13">
+        <v>6</v>
+      </c>
+      <c r="J13">
+        <v>10</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>6</v>
+      </c>
+      <c r="O13">
+        <v>0</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>30</v>
+      </c>
+      <c r="AF13" t="str">
+        <v>Parn photo 01M59J9W15MTJBBSM3HW27H67W.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Grape 3, Mangosteen 3, Pomegranate 2 | CHECK: branch written "B-5"</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>11/10/2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C14">
+        <v>3171</v>
+      </c>
+      <c r="D14">
+        <v>1855</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>1316</v>
+      </c>
+      <c r="H14">
+        <v>8</v>
+      </c>
+      <c r="J14">
+        <v>13</v>
+      </c>
+      <c r="K14">
+        <v>1</v>
+      </c>
+      <c r="M14">
+        <v>4</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>38</v>
+      </c>
+      <c r="AF14" t="str">
+        <v>Parn photo 01M59J9JG37K1VYNWM1E9HNJYM.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 8, Pomegranate 2, Grape 2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C15">
+        <v>1309</v>
+      </c>
+      <c r="D15">
+        <v>409</v>
+      </c>
+      <c r="E15">
+        <v>60</v>
+      </c>
+      <c r="G15">
+        <v>900</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15">
+        <v>5</v>
+      </c>
+      <c r="K15">
+        <v>2</v>
+      </c>
+      <c r="M15">
+        <v>2</v>
+      </c>
+      <c r="O15">
+        <v>2</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>16</v>
+      </c>
+      <c r="AF15" t="str">
+        <v>Parn photo 01M59J9QSHRE98Q4HPM1DFAWG2.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Pomegranate 2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>13/10/2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C16">
+        <v>1787</v>
+      </c>
+      <c r="D16">
+        <v>1269</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>518</v>
+      </c>
+      <c r="H16">
+        <v>2</v>
+      </c>
+      <c r="J16">
+        <v>4</v>
+      </c>
+      <c r="K16">
+        <v>2</v>
+      </c>
+      <c r="M16">
+        <v>1</v>
+      </c>
+      <c r="O16">
+        <v>2</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>20</v>
+      </c>
+      <c r="AF16" t="str">
+        <v>Parn photo 01M59J9QWVD64QHPK4D8GBFXW2.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 2, Pomegranate 3, Grape 3, Pear 1 | CHECK: price assumed: Pear 60 (no price written)</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>14/10/2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C17">
+        <v>1298</v>
+      </c>
+      <c r="D17">
+        <v>1178</v>
+      </c>
+      <c r="E17">
+        <v>60</v>
+      </c>
+      <c r="G17">
+        <v>120</v>
+      </c>
+      <c r="H17">
+        <v>4</v>
+      </c>
+      <c r="J17">
+        <v>5</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>2</v>
+      </c>
+      <c r="O17">
+        <v>2</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>17</v>
+      </c>
+      <c r="AF17" t="str">
+        <v>Parn photo 01M59J9R227FMK8RSXAKR7E6M5.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 2, Pomegranate 1, Grape 1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>15/10/2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C18">
+        <v>1916</v>
+      </c>
+      <c r="D18">
+        <v>1388</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>528</v>
+      </c>
+      <c r="H18">
+        <v>4</v>
+      </c>
+      <c r="J18">
+        <v>4</v>
+      </c>
+      <c r="K18">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>5</v>
+      </c>
+      <c r="O18">
+        <v>3</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+      <c r="Q18">
+        <v>23</v>
+      </c>
+      <c r="AF18" t="str">
+        <v>Parn photo 01M59J9R6FFZ1CKESJ3KWJVWNK.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 3, Grape 1, Pomegranate 2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>16/10/2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C19">
+        <v>1437</v>
+      </c>
+      <c r="D19">
+        <v>618</v>
+      </c>
+      <c r="E19">
+        <v>60</v>
+      </c>
+      <c r="G19">
+        <v>819</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
+      </c>
+      <c r="J19">
+        <v>6</v>
+      </c>
+      <c r="K19">
+        <v>2</v>
+      </c>
+      <c r="M19">
+        <v>1</v>
+      </c>
+      <c r="O19">
+        <v>1</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>16</v>
+      </c>
+      <c r="AF19" t="str">
+        <v>Parn photo 01M59J9VECNZD8JCVTAZKJQ4QT.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 3, Pomegranate 2 | CHECK: sheet totals are after ice (cash 558, grand 1377); ice 60 added back</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>17/10/2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C20">
+        <v>907</v>
+      </c>
+      <c r="D20">
+        <v>439</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>468</v>
+      </c>
+      <c r="H20">
+        <v>3</v>
+      </c>
+      <c r="J20">
+        <v>3</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="M20">
+        <v>2</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>10</v>
+      </c>
+      <c r="AF20" t="str">
+        <v>Parn photo 01M59J9R6H13PYS5JQN9Y3C7KJ.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 1, Pomegranate 1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>18/10/2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C21">
+        <v>1786</v>
+      </c>
+      <c r="D21">
+        <v>1257</v>
+      </c>
+      <c r="E21">
+        <v>60</v>
+      </c>
+      <c r="G21">
+        <v>529</v>
+      </c>
+      <c r="H21">
+        <v>3</v>
+      </c>
+      <c r="J21">
+        <v>1</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="M21">
+        <v>5</v>
+      </c>
+      <c r="O21">
+        <v>1</v>
+      </c>
+      <c r="P21">
+        <v>0</v>
+      </c>
+      <c r="Q21">
+        <v>19</v>
+      </c>
+      <c r="AF21" t="str">
+        <v>Parn photo 01M59J9RT4N01RJ9EQEA7BH6K3.jpg (B4 Oct26 Daily Sales Record, undated sheet) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Pomegranate 3, Grape 3, Mangosteen 3 | CHECK: UNDATED sheet booked as 18/10/2026 on Parn's word; branch written "blank"; Parn 19/10/2026: undated sheet is 18 Oct</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AF3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
B4 Mangosteen column; LINE bot knows all branches and all published months (approved by Parn)
B4 Sep26-Dec26: new Mangosteen + Mangosteen (฿) columns. Sep mangosteen moved out of Mango (34 cups, 4386); Oct 75 cups, 9726. Revenue/cash/scan/exp/Total Cups unchanged (Sep 12,435, Oct 43,100). Bot owner note: all branches B1-B4, every published day from the live data.json (was last 14 days, B1-B3 only). B4/B-04/B-5 read as B4 in the photo flow; bot commit includes the B4 workbook.
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B4_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B4_2026.xlsx
@@ -134,10 +134,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -169,10 +169,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -426,7 +426,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF13"/>
+  <dimension ref="A1:AH13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -483,51 +483,57 @@
         <v>Pineapple</v>
       </c>
       <c r="Q3" t="str">
+        <v>Mangosteen</v>
+      </c>
+      <c r="R3" t="str">
+        <v>Mangosteen (฿)</v>
+      </c>
+      <c r="S3" t="str">
         <v>Total Cups</v>
       </c>
-      <c r="R3" t="str">
+      <c r="T3" t="str">
         <v>Bot Big</v>
       </c>
-      <c r="S3" t="str">
+      <c r="U3" t="str">
         <v>Bot Small</v>
       </c>
-      <c r="T3" t="str">
+      <c r="V3" t="str">
         <v>Used Orange (basket)</v>
       </c>
-      <c r="U3" t="str">
+      <c r="W3" t="str">
         <v>Used Watermelon (pcs)</v>
       </c>
-      <c r="V3" t="str">
+      <c r="X3" t="str">
         <v>Used Mango</v>
       </c>
-      <c r="W3" t="str">
+      <c r="Y3" t="str">
         <v>Used Coco (Meat)</v>
       </c>
-      <c r="X3" t="str">
+      <c r="Z3" t="str">
         <v>Used Coco (Water)</v>
       </c>
-      <c r="Y3" t="str">
+      <c r="AA3" t="str">
         <v>Used Coco (Conden)</v>
       </c>
-      <c r="Z3" t="str">
+      <c r="AB3" t="str">
         <v>Used Coco (Raw)</v>
       </c>
-      <c r="AA3" t="str">
+      <c r="AC3" t="str">
         <v>Used Apple</v>
       </c>
-      <c r="AB3" t="str">
+      <c r="AD3" t="str">
         <v>Used Guava</v>
       </c>
-      <c r="AC3" t="str">
+      <c r="AE3" t="str">
         <v>Used Pineapple</v>
       </c>
-      <c r="AD3" t="str">
+      <c r="AF3" t="str">
         <v>Used Young Coco</v>
       </c>
-      <c r="AE3" t="str">
+      <c r="AG3" t="str">
         <v>Bottle Revenue (฿)</v>
       </c>
-      <c r="AF3" t="str">
+      <c r="AH3" t="str">
         <v>Source Note</v>
       </c>
     </row>
@@ -581,26 +587,26 @@
         <v>0</v>
       </c>
       <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
         <v>4</v>
       </c>
-      <c r="R4">
-        <v>0</v>
-      </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
       <c r="T4">
         <v>0</v>
       </c>
       <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
         <v>4</v>
       </c>
-      <c r="V4">
-        <v>0</v>
-      </c>
-      <c r="W4">
-        <v>0</v>
-      </c>
       <c r="X4">
         <v>0</v>
       </c>
@@ -625,7 +631,13 @@
       <c r="AE4">
         <v>0</v>
       </c>
-      <c r="AF4" t="str">
+      <c r="AF4">
+        <v>0</v>
+      </c>
+      <c r="AG4">
+        <v>0</v>
+      </c>
+      <c r="AH4" t="str">
         <v>LINE_ALBUM_Sales for September (B-4)_261002_9.jpg</v>
       </c>
     </row>
@@ -661,7 +673,7 @@
         <v>2</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -679,29 +691,29 @@
         <v>0</v>
       </c>
       <c r="Q5">
+        <v>1</v>
+      </c>
+      <c r="R5">
+        <v>129</v>
+      </c>
+      <c r="S5">
         <v>4</v>
       </c>
-      <c r="R5">
-        <v>0</v>
-      </c>
-      <c r="S5">
-        <v>0</v>
-      </c>
       <c r="T5">
         <v>0</v>
       </c>
       <c r="U5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>2</v>
+      </c>
+      <c r="X5">
         <v>1</v>
       </c>
-      <c r="W5">
-        <v>0</v>
-      </c>
-      <c r="X5">
-        <v>0</v>
-      </c>
       <c r="Y5">
         <v>0</v>
       </c>
@@ -709,21 +721,27 @@
         <v>0</v>
       </c>
       <c r="AA5">
+        <v>0</v>
+      </c>
+      <c r="AB5">
+        <v>0</v>
+      </c>
+      <c r="AC5">
         <v>1</v>
       </c>
-      <c r="AB5">
-        <v>0</v>
-      </c>
-      <c r="AC5">
-        <v>0</v>
-      </c>
       <c r="AD5">
         <v>0</v>
       </c>
       <c r="AE5">
         <v>0</v>
       </c>
-      <c r="AF5" t="str">
+      <c r="AF5">
+        <v>0</v>
+      </c>
+      <c r="AG5">
+        <v>0</v>
+      </c>
+      <c r="AH5" t="str">
         <v>LINE_ALBUM_Sales for September (B-4)_261002_10.jpg</v>
       </c>
     </row>
@@ -759,7 +777,7 @@
         <v>1</v>
       </c>
       <c r="K6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -777,28 +795,28 @@
         <v>0</v>
       </c>
       <c r="Q6">
+        <v>2</v>
+      </c>
+      <c r="R6">
+        <v>258</v>
+      </c>
+      <c r="S6">
         <v>6</v>
       </c>
-      <c r="R6">
-        <v>0</v>
-      </c>
-      <c r="S6">
-        <v>0</v>
-      </c>
       <c r="T6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>2</v>
+      </c>
+      <c r="W6">
         <v>1</v>
       </c>
-      <c r="V6">
-        <v>2</v>
-      </c>
-      <c r="W6">
-        <v>0</v>
-      </c>
       <c r="X6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y6">
         <v>0</v>
@@ -807,21 +825,27 @@
         <v>0</v>
       </c>
       <c r="AA6">
+        <v>0</v>
+      </c>
+      <c r="AB6">
+        <v>0</v>
+      </c>
+      <c r="AC6">
         <v>1</v>
       </c>
-      <c r="AB6">
-        <v>0</v>
-      </c>
-      <c r="AC6">
-        <v>0</v>
-      </c>
       <c r="AD6">
         <v>0</v>
       </c>
       <c r="AE6">
         <v>0</v>
       </c>
-      <c r="AF6" t="str">
+      <c r="AF6">
+        <v>0</v>
+      </c>
+      <c r="AG6">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="str">
         <v>LINE_ALBUM_Sales for September (B-4)_261002_11.jpg</v>
       </c>
     </row>
@@ -857,7 +881,7 @@
         <v>7</v>
       </c>
       <c r="K7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -875,28 +899,28 @@
         <v>0</v>
       </c>
       <c r="Q7">
+        <v>2</v>
+      </c>
+      <c r="R7">
+        <v>258</v>
+      </c>
+      <c r="S7">
         <v>12</v>
       </c>
-      <c r="R7">
-        <v>0</v>
-      </c>
-      <c r="S7">
-        <v>0</v>
-      </c>
       <c r="T7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U7">
+        <v>0</v>
+      </c>
+      <c r="V7">
+        <v>2</v>
+      </c>
+      <c r="W7">
         <v>7</v>
       </c>
-      <c r="V7">
-        <v>2</v>
-      </c>
-      <c r="W7">
-        <v>0</v>
-      </c>
       <c r="X7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y7">
         <v>0</v>
@@ -905,21 +929,27 @@
         <v>0</v>
       </c>
       <c r="AA7">
+        <v>0</v>
+      </c>
+      <c r="AB7">
+        <v>0</v>
+      </c>
+      <c r="AC7">
         <v>1</v>
       </c>
-      <c r="AB7">
-        <v>0</v>
-      </c>
-      <c r="AC7">
-        <v>0</v>
-      </c>
       <c r="AD7">
         <v>0</v>
       </c>
       <c r="AE7">
         <v>0</v>
       </c>
-      <c r="AF7" t="str">
+      <c r="AF7">
+        <v>0</v>
+      </c>
+      <c r="AG7">
+        <v>0</v>
+      </c>
+      <c r="AH7" t="str">
         <v>LINE_ALBUM_Sales for September (B-4)_261002_8.jpg</v>
       </c>
     </row>
@@ -955,7 +985,7 @@
         <v>8</v>
       </c>
       <c r="K8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L8">
         <v>0</v>
@@ -973,29 +1003,29 @@
         <v>0</v>
       </c>
       <c r="Q8">
+        <v>4</v>
+      </c>
+      <c r="R8">
+        <v>516</v>
+      </c>
+      <c r="S8">
         <v>15</v>
       </c>
-      <c r="R8">
-        <v>0</v>
-      </c>
-      <c r="S8">
-        <v>0</v>
-      </c>
       <c r="T8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>2</v>
+      </c>
+      <c r="W8">
         <v>8</v>
       </c>
-      <c r="V8">
+      <c r="X8">
         <v>4</v>
       </c>
-      <c r="W8">
-        <v>0</v>
-      </c>
-      <c r="X8">
-        <v>0</v>
-      </c>
       <c r="Y8">
         <v>0</v>
       </c>
@@ -1003,21 +1033,27 @@
         <v>0</v>
       </c>
       <c r="AA8">
+        <v>0</v>
+      </c>
+      <c r="AB8">
+        <v>0</v>
+      </c>
+      <c r="AC8">
         <v>1</v>
       </c>
-      <c r="AB8">
-        <v>0</v>
-      </c>
-      <c r="AC8">
-        <v>0</v>
-      </c>
       <c r="AD8">
         <v>0</v>
       </c>
       <c r="AE8">
         <v>0</v>
       </c>
-      <c r="AF8" t="str">
+      <c r="AF8">
+        <v>0</v>
+      </c>
+      <c r="AG8">
+        <v>0</v>
+      </c>
+      <c r="AH8" t="str">
         <v>LINE_ALBUM_Sales for September (B-4)_261002_7.jpg</v>
       </c>
     </row>
@@ -1053,47 +1089,47 @@
         <v>1</v>
       </c>
       <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>2</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
         <v>1</v>
       </c>
-      <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9">
-        <v>2</v>
-      </c>
-      <c r="N9">
-        <v>0</v>
-      </c>
-      <c r="O9">
-        <v>0</v>
-      </c>
-      <c r="P9">
-        <v>0</v>
-      </c>
-      <c r="Q9">
+      <c r="R9">
+        <v>129</v>
+      </c>
+      <c r="S9">
         <v>4</v>
       </c>
-      <c r="R9">
-        <v>0</v>
-      </c>
-      <c r="S9">
-        <v>0</v>
-      </c>
       <c r="T9">
         <v>0</v>
       </c>
       <c r="U9">
+        <v>0</v>
+      </c>
+      <c r="V9">
+        <v>0</v>
+      </c>
+      <c r="W9">
         <v>1</v>
       </c>
-      <c r="V9">
+      <c r="X9">
         <v>1</v>
       </c>
-      <c r="W9">
-        <v>0</v>
-      </c>
-      <c r="X9">
-        <v>0</v>
-      </c>
       <c r="Y9">
         <v>0</v>
       </c>
@@ -1101,13 +1137,13 @@
         <v>0</v>
       </c>
       <c r="AA9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AB9">
         <v>0</v>
       </c>
       <c r="AC9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD9">
         <v>0</v>
@@ -1115,7 +1151,13 @@
       <c r="AE9">
         <v>0</v>
       </c>
-      <c r="AF9" t="str">
+      <c r="AF9">
+        <v>0</v>
+      </c>
+      <c r="AG9">
+        <v>0</v>
+      </c>
+      <c r="AH9" t="str">
         <v>LINE_ALBUM_Sales for September (B-4)_261002_5.jpg</v>
       </c>
     </row>
@@ -1151,7 +1193,7 @@
         <v>4</v>
       </c>
       <c r="K10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L10">
         <v>0</v>
@@ -1169,28 +1211,28 @@
         <v>0</v>
       </c>
       <c r="Q10">
+        <v>4</v>
+      </c>
+      <c r="R10">
+        <v>516</v>
+      </c>
+      <c r="S10">
         <v>17</v>
       </c>
-      <c r="R10">
-        <v>0</v>
-      </c>
-      <c r="S10">
-        <v>0</v>
-      </c>
       <c r="T10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="U10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V10">
         <v>4</v>
       </c>
       <c r="W10">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X10">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Y10">
         <v>0</v>
@@ -1199,21 +1241,27 @@
         <v>0</v>
       </c>
       <c r="AA10">
+        <v>0</v>
+      </c>
+      <c r="AB10">
+        <v>0</v>
+      </c>
+      <c r="AC10">
         <v>4</v>
       </c>
-      <c r="AB10">
+      <c r="AD10">
         <v>1</v>
       </c>
-      <c r="AC10">
-        <v>0</v>
-      </c>
-      <c r="AD10">
-        <v>0</v>
-      </c>
       <c r="AE10">
         <v>0</v>
       </c>
-      <c r="AF10" t="str">
+      <c r="AF10">
+        <v>0</v>
+      </c>
+      <c r="AG10">
+        <v>0</v>
+      </c>
+      <c r="AH10" t="str">
         <v>LINE_ALBUM_Sales for September (B-4)_261002_4.jpg</v>
       </c>
     </row>
@@ -1249,7 +1297,7 @@
         <v>7</v>
       </c>
       <c r="K11">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -1267,29 +1315,29 @@
         <v>0</v>
       </c>
       <c r="Q11">
+        <v>7</v>
+      </c>
+      <c r="R11">
+        <v>903</v>
+      </c>
+      <c r="S11">
         <v>29</v>
       </c>
-      <c r="R11">
-        <v>0</v>
-      </c>
-      <c r="S11">
-        <v>0</v>
-      </c>
       <c r="T11">
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <v>0</v>
+      </c>
+      <c r="V11">
         <v>7</v>
       </c>
-      <c r="U11">
+      <c r="W11">
         <v>7</v>
       </c>
-      <c r="V11">
+      <c r="X11">
         <v>11</v>
       </c>
-      <c r="W11">
-        <v>0</v>
-      </c>
-      <c r="X11">
-        <v>0</v>
-      </c>
       <c r="Y11">
         <v>0</v>
       </c>
@@ -1297,21 +1345,27 @@
         <v>0</v>
       </c>
       <c r="AA11">
+        <v>0</v>
+      </c>
+      <c r="AB11">
+        <v>0</v>
+      </c>
+      <c r="AC11">
         <v>1</v>
       </c>
-      <c r="AB11">
+      <c r="AD11">
         <v>3</v>
       </c>
-      <c r="AC11">
-        <v>0</v>
-      </c>
-      <c r="AD11">
-        <v>0</v>
-      </c>
       <c r="AE11">
         <v>0</v>
       </c>
-      <c r="AF11" t="str">
+      <c r="AF11">
+        <v>0</v>
+      </c>
+      <c r="AG11">
+        <v>0</v>
+      </c>
+      <c r="AH11" t="str">
         <v>LINE_ALBUM_Sales for September (B-4)_261002_3.jpg</v>
       </c>
     </row>
@@ -1347,7 +1401,7 @@
         <v>6</v>
       </c>
       <c r="K12">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -1365,29 +1419,29 @@
         <v>0</v>
       </c>
       <c r="Q12">
+        <v>8</v>
+      </c>
+      <c r="R12">
+        <v>1032</v>
+      </c>
+      <c r="S12">
         <v>23</v>
       </c>
-      <c r="R12">
-        <v>0</v>
-      </c>
-      <c r="S12">
-        <v>0</v>
-      </c>
       <c r="T12">
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <v>0</v>
+      </c>
+      <c r="V12">
         <v>5</v>
       </c>
-      <c r="U12">
+      <c r="W12">
         <v>6</v>
       </c>
-      <c r="V12">
+      <c r="X12">
         <v>8</v>
       </c>
-      <c r="W12">
-        <v>0</v>
-      </c>
-      <c r="X12">
-        <v>0</v>
-      </c>
       <c r="Y12">
         <v>0</v>
       </c>
@@ -1395,21 +1449,27 @@
         <v>0</v>
       </c>
       <c r="AA12">
+        <v>0</v>
+      </c>
+      <c r="AB12">
+        <v>0</v>
+      </c>
+      <c r="AC12">
         <v>4</v>
       </c>
-      <c r="AB12">
-        <v>0</v>
-      </c>
-      <c r="AC12">
-        <v>0</v>
-      </c>
       <c r="AD12">
         <v>0</v>
       </c>
       <c r="AE12">
         <v>0</v>
       </c>
-      <c r="AF12" t="str">
+      <c r="AF12">
+        <v>0</v>
+      </c>
+      <c r="AG12">
+        <v>0</v>
+      </c>
+      <c r="AH12" t="str">
         <v>LINE_ALBUM_Sales for September (B-4)_261002_2.jpg</v>
       </c>
     </row>
@@ -1445,7 +1505,7 @@
         <v>9</v>
       </c>
       <c r="K13">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L13">
         <v>5</v>
@@ -1463,64 +1523,70 @@
         <v>0</v>
       </c>
       <c r="Q13">
+        <v>5</v>
+      </c>
+      <c r="R13">
+        <v>645</v>
+      </c>
+      <c r="S13">
         <v>29</v>
       </c>
-      <c r="R13">
-        <v>0</v>
-      </c>
-      <c r="S13">
-        <v>0</v>
-      </c>
       <c r="T13">
+        <v>0</v>
+      </c>
+      <c r="U13">
+        <v>0</v>
+      </c>
+      <c r="V13">
         <v>6</v>
       </c>
-      <c r="U13">
+      <c r="W13">
         <v>9</v>
       </c>
-      <c r="V13">
+      <c r="X13">
         <v>7</v>
       </c>
-      <c r="W13">
-        <v>0</v>
-      </c>
-      <c r="X13">
-        <v>0</v>
-      </c>
       <c r="Y13">
         <v>0</v>
       </c>
       <c r="Z13">
+        <v>0</v>
+      </c>
+      <c r="AA13">
+        <v>0</v>
+      </c>
+      <c r="AB13">
         <v>5</v>
       </c>
-      <c r="AA13">
+      <c r="AC13">
         <v>1</v>
       </c>
-      <c r="AB13">
+      <c r="AD13">
         <v>1</v>
       </c>
-      <c r="AC13">
-        <v>0</v>
-      </c>
-      <c r="AD13">
-        <v>0</v>
-      </c>
       <c r="AE13">
         <v>0</v>
       </c>
-      <c r="AF13" t="str">
+      <c r="AF13">
+        <v>0</v>
+      </c>
+      <c r="AG13">
+        <v>0</v>
+      </c>
+      <c r="AH13" t="str">
         <v>LINE_ALBUM_Sales for September (B-4)_261002_1.jpg</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AF13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF21"/>
+  <dimension ref="A1:AH21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1577,51 +1643,57 @@
         <v>Pineapple</v>
       </c>
       <c r="Q3" t="str">
+        <v>Mangosteen</v>
+      </c>
+      <c r="R3" t="str">
+        <v>Mangosteen (฿)</v>
+      </c>
+      <c r="S3" t="str">
         <v>Total Cups</v>
       </c>
-      <c r="R3" t="str">
+      <c r="T3" t="str">
         <v>Bot Big</v>
       </c>
-      <c r="S3" t="str">
+      <c r="U3" t="str">
         <v>Bot Small</v>
       </c>
-      <c r="T3" t="str">
+      <c r="V3" t="str">
         <v>Used Orange (basket)</v>
       </c>
-      <c r="U3" t="str">
+      <c r="W3" t="str">
         <v>Used Watermelon (pcs)</v>
       </c>
-      <c r="V3" t="str">
+      <c r="X3" t="str">
         <v>Used Mango</v>
       </c>
-      <c r="W3" t="str">
+      <c r="Y3" t="str">
         <v>Used Coco (Meat)</v>
       </c>
-      <c r="X3" t="str">
+      <c r="Z3" t="str">
         <v>Used Coco (Water)</v>
       </c>
-      <c r="Y3" t="str">
+      <c r="AA3" t="str">
         <v>Used Coco (Conden)</v>
       </c>
-      <c r="Z3" t="str">
+      <c r="AB3" t="str">
         <v>Used Coco (Raw)</v>
       </c>
-      <c r="AA3" t="str">
+      <c r="AC3" t="str">
         <v>Used Apple</v>
       </c>
-      <c r="AB3" t="str">
+      <c r="AD3" t="str">
         <v>Used Guava</v>
       </c>
-      <c r="AC3" t="str">
+      <c r="AE3" t="str">
         <v>Used Pineapple</v>
       </c>
-      <c r="AD3" t="str">
+      <c r="AF3" t="str">
         <v>Used Young Coco</v>
       </c>
-      <c r="AE3" t="str">
+      <c r="AG3" t="str">
         <v>Bottle Revenue (฿)</v>
       </c>
-      <c r="AF3" t="str">
+      <c r="AH3" t="str">
         <v>Source Note</v>
       </c>
     </row>
@@ -1663,9 +1735,15 @@
         <v>2</v>
       </c>
       <c r="Q4">
+        <v>10</v>
+      </c>
+      <c r="R4">
+        <v>1290</v>
+      </c>
+      <c r="S4">
         <v>46</v>
       </c>
-      <c r="AF4" t="str">
+      <c r="AH4" t="str">
         <v>Parn photo 01M59J90GR140C7NWESP7HBDJE.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 10, Pomegranate 2 | CHECK: branch written "B-5"</v>
       </c>
     </row>
@@ -1707,9 +1785,15 @@
         <v>2</v>
       </c>
       <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
         <v>49</v>
       </c>
-      <c r="AF5" t="str">
+      <c r="AH5" t="str">
         <v>Parn photo 01M59J91CQJHZ1H6GQWYSH15T0.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Pomegranate 11 | CHECK: branch written "blank"</v>
       </c>
     </row>
@@ -1751,9 +1835,15 @@
         <v>4</v>
       </c>
       <c r="Q6">
+        <v>10</v>
+      </c>
+      <c r="R6">
+        <v>1290</v>
+      </c>
+      <c r="S6">
         <v>56</v>
       </c>
-      <c r="AF6" t="str">
+      <c r="AH6" t="str">
         <v>Parn photo 01M59J91CE83KN64KME60GJ66C.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 10, Grape 4, Pomegranate 5 | CHECK: branch written "B-5"</v>
       </c>
     </row>
@@ -1795,9 +1885,15 @@
         <v>3</v>
       </c>
       <c r="Q7">
+        <v>10</v>
+      </c>
+      <c r="R7">
+        <v>1341</v>
+      </c>
+      <c r="S7">
         <v>51</v>
       </c>
-      <c r="AF7" t="str">
+      <c r="AH7" t="str">
         <v>Parn photo 01M59J9S2F8Z1WNM683T3F3ZER.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 9, Grape 4, Pomegranate 5, Mangosteen no ice 1 | CHECK: cash items 2511 vs written 2691 (+180); branch written "B-5"</v>
       </c>
     </row>
@@ -1842,9 +1938,15 @@
         <v>0</v>
       </c>
       <c r="Q8">
+        <v>8</v>
+      </c>
+      <c r="R8">
+        <v>1032</v>
+      </c>
+      <c r="S8">
         <v>30</v>
       </c>
-      <c r="AF8" t="str">
+      <c r="AH8" t="str">
         <v>Parn photo 01M59J91AM9M9BMFPWVR3PJFEJ.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 8, Grape 2, Pomegranate 3 | CHECK: branch written "B-5"</v>
       </c>
     </row>
@@ -1886,9 +1988,15 @@
         <v>0</v>
       </c>
       <c r="Q9">
+        <v>2</v>
+      </c>
+      <c r="R9">
+        <v>258</v>
+      </c>
+      <c r="S9">
         <v>14</v>
       </c>
-      <c r="AF9" t="str">
+      <c r="AH9" t="str">
         <v>Parn photo 01M59J9K44G95R8NMDKVV135ZR.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 2, Grape 1, Pomegranate 1 | CHECK: branch written "B-5"</v>
       </c>
     </row>
@@ -1930,9 +2038,15 @@
         <v>0</v>
       </c>
       <c r="Q10">
+        <v>2</v>
+      </c>
+      <c r="R10">
+        <v>258</v>
+      </c>
+      <c r="S10">
         <v>19</v>
       </c>
-      <c r="AF10" t="str">
+      <c r="AH10" t="str">
         <v>Parn photo 01M59J9NN1659SB4KXXHTQHHYN.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 2, Pomegranate 1 | CHECK: branch written "B-04"</v>
       </c>
     </row>
@@ -1974,9 +2088,15 @@
         <v>0</v>
       </c>
       <c r="Q11">
+        <v>4</v>
+      </c>
+      <c r="R11">
+        <v>516</v>
+      </c>
+      <c r="S11">
         <v>23</v>
       </c>
-      <c r="AF11" t="str">
+      <c r="AH11" t="str">
         <v>Parn photo 01M59J91C84W60ZV60XAC5R6V3.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 4, Pomegranate 2, Grape 4 | CHECK: cash items 1089 vs booked 1086 (-3); branch written "B-04"; ice 60 written then crossed out; Parn 19/10/2026: book written grand total 1963 (not 1966); 3 taken off cash (1089 -&gt; 1086), QR 877 unchanged</v>
       </c>
     </row>
@@ -2018,9 +2138,15 @@
         <v>0</v>
       </c>
       <c r="Q12">
+        <v>4</v>
+      </c>
+      <c r="R12">
+        <v>516</v>
+      </c>
+      <c r="S12">
         <v>15</v>
       </c>
-      <c r="AF12" t="str">
+      <c r="AH12" t="str">
         <v>Parn photo 01M59J91D2ZT3CV2DWW9GJGHC0.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 4, Pomegranate 1, Grape 1 | CHECK: no grand total written; cash 886 + QR 360 = 1246; branch written "B-04"</v>
       </c>
     </row>
@@ -2062,9 +2188,15 @@
         <v>0</v>
       </c>
       <c r="Q13">
+        <v>3</v>
+      </c>
+      <c r="R13">
+        <v>387</v>
+      </c>
+      <c r="S13">
         <v>30</v>
       </c>
-      <c r="AF13" t="str">
+      <c r="AH13" t="str">
         <v>Parn photo 01M59J9W15MTJBBSM3HW27H67W.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Grape 3, Mangosteen 3, Pomegranate 2 | CHECK: branch written "B-5"</v>
       </c>
     </row>
@@ -2106,9 +2238,15 @@
         <v>0</v>
       </c>
       <c r="Q14">
+        <v>8</v>
+      </c>
+      <c r="R14">
+        <v>1032</v>
+      </c>
+      <c r="S14">
         <v>38</v>
       </c>
-      <c r="AF14" t="str">
+      <c r="AH14" t="str">
         <v>Parn photo 01M59J9JG37K1VYNWM1E9HNJYM.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 8, Pomegranate 2, Grape 2</v>
       </c>
     </row>
@@ -2153,9 +2291,15 @@
         <v>0</v>
       </c>
       <c r="Q15">
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15">
         <v>16</v>
       </c>
-      <c r="AF15" t="str">
+      <c r="AH15" t="str">
         <v>Parn photo 01M59J9QSHRE98Q4HPM1DFAWG2.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Pomegranate 2</v>
       </c>
     </row>
@@ -2197,9 +2341,15 @@
         <v>0</v>
       </c>
       <c r="Q16">
+        <v>2</v>
+      </c>
+      <c r="R16">
+        <v>258</v>
+      </c>
+      <c r="S16">
         <v>20</v>
       </c>
-      <c r="AF16" t="str">
+      <c r="AH16" t="str">
         <v>Parn photo 01M59J9QWVD64QHPK4D8GBFXW2.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 2, Pomegranate 3, Grape 3, Pear 1 | CHECK: price assumed: Pear 60 (no price written)</v>
       </c>
     </row>
@@ -2241,9 +2391,15 @@
         <v>0</v>
       </c>
       <c r="Q17">
+        <v>2</v>
+      </c>
+      <c r="R17">
+        <v>258</v>
+      </c>
+      <c r="S17">
         <v>17</v>
       </c>
-      <c r="AF17" t="str">
+      <c r="AH17" t="str">
         <v>Parn photo 01M59J9R227FMK8RSXAKR7E6M5.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 2, Pomegranate 1, Grape 1</v>
       </c>
     </row>
@@ -2285,9 +2441,15 @@
         <v>0</v>
       </c>
       <c r="Q18">
+        <v>3</v>
+      </c>
+      <c r="R18">
+        <v>387</v>
+      </c>
+      <c r="S18">
         <v>23</v>
       </c>
-      <c r="AF18" t="str">
+      <c r="AH18" t="str">
         <v>Parn photo 01M59J9R6FFZ1CKESJ3KWJVWNK.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 3, Grape 1, Pomegranate 2</v>
       </c>
     </row>
@@ -2329,9 +2491,15 @@
         <v>0</v>
       </c>
       <c r="Q19">
+        <v>3</v>
+      </c>
+      <c r="R19">
+        <v>387</v>
+      </c>
+      <c r="S19">
         <v>16</v>
       </c>
-      <c r="AF19" t="str">
+      <c r="AH19" t="str">
         <v>Parn photo 01M59J9VECNZD8JCVTAZKJQ4QT.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 3, Pomegranate 2 | CHECK: sheet totals are after ice (cash 558, grand 1377); ice 60 added back</v>
       </c>
     </row>
@@ -2373,9 +2541,15 @@
         <v>0</v>
       </c>
       <c r="Q20">
+        <v>1</v>
+      </c>
+      <c r="R20">
+        <v>129</v>
+      </c>
+      <c r="S20">
         <v>10</v>
       </c>
-      <c r="AF20" t="str">
+      <c r="AH20" t="str">
         <v>Parn photo 01M59J9R6H13PYS5JQN9Y3C7KJ.jpg (B4 Oct26 Daily Sales Record) | before ice; ice 0 in Expenses | not in fruit columns (in Total Cups only): Mangosteen 1, Pomegranate 1</v>
       </c>
     </row>
@@ -2417,22 +2591,28 @@
         <v>0</v>
       </c>
       <c r="Q21">
+        <v>3</v>
+      </c>
+      <c r="R21">
+        <v>387</v>
+      </c>
+      <c r="S21">
         <v>19</v>
       </c>
-      <c r="AF21" t="str">
+      <c r="AH21" t="str">
         <v>Parn photo 01M59J9RT4N01RJ9EQEA7BH6K3.jpg (B4 Oct26 Daily Sales Record, undated sheet) | before ice; ice 60 in Expenses | not in fruit columns (in Total Cups only): Pomegranate 3, Grape 3, Mangosteen 3 | CHECK: UNDATED sheet booked as 18/10/2026 on Parn's word; branch written "blank"; Parn 19/10/2026: undated sheet is 18 Oct</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AF21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH21"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF3"/>
+  <dimension ref="A1:AH3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2489,64 +2669,70 @@
         <v>Pineapple</v>
       </c>
       <c r="Q3" t="str">
+        <v>Mangosteen</v>
+      </c>
+      <c r="R3" t="str">
+        <v>Mangosteen (฿)</v>
+      </c>
+      <c r="S3" t="str">
         <v>Total Cups</v>
       </c>
-      <c r="R3" t="str">
+      <c r="T3" t="str">
         <v>Bot Big</v>
       </c>
-      <c r="S3" t="str">
+      <c r="U3" t="str">
         <v>Bot Small</v>
       </c>
-      <c r="T3" t="str">
+      <c r="V3" t="str">
         <v>Used Orange (basket)</v>
       </c>
-      <c r="U3" t="str">
+      <c r="W3" t="str">
         <v>Used Watermelon (pcs)</v>
       </c>
-      <c r="V3" t="str">
+      <c r="X3" t="str">
         <v>Used Mango</v>
       </c>
-      <c r="W3" t="str">
+      <c r="Y3" t="str">
         <v>Used Coco (Meat)</v>
       </c>
-      <c r="X3" t="str">
+      <c r="Z3" t="str">
         <v>Used Coco (Water)</v>
       </c>
-      <c r="Y3" t="str">
+      <c r="AA3" t="str">
         <v>Used Coco (Conden)</v>
       </c>
-      <c r="Z3" t="str">
+      <c r="AB3" t="str">
         <v>Used Coco (Raw)</v>
       </c>
-      <c r="AA3" t="str">
+      <c r="AC3" t="str">
         <v>Used Apple</v>
       </c>
-      <c r="AB3" t="str">
+      <c r="AD3" t="str">
         <v>Used Guava</v>
       </c>
-      <c r="AC3" t="str">
+      <c r="AE3" t="str">
         <v>Used Pineapple</v>
       </c>
-      <c r="AD3" t="str">
+      <c r="AF3" t="str">
         <v>Used Young Coco</v>
       </c>
-      <c r="AE3" t="str">
+      <c r="AG3" t="str">
         <v>Bottle Revenue (฿)</v>
       </c>
-      <c r="AF3" t="str">
+      <c r="AH3" t="str">
         <v>Source Note</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AF3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF3"/>
+  <dimension ref="A1:AH3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2603,57 +2789,63 @@
         <v>Pineapple</v>
       </c>
       <c r="Q3" t="str">
+        <v>Mangosteen</v>
+      </c>
+      <c r="R3" t="str">
+        <v>Mangosteen (฿)</v>
+      </c>
+      <c r="S3" t="str">
         <v>Total Cups</v>
       </c>
-      <c r="R3" t="str">
+      <c r="T3" t="str">
         <v>Bot Big</v>
       </c>
-      <c r="S3" t="str">
+      <c r="U3" t="str">
         <v>Bot Small</v>
       </c>
-      <c r="T3" t="str">
+      <c r="V3" t="str">
         <v>Used Orange (basket)</v>
       </c>
-      <c r="U3" t="str">
+      <c r="W3" t="str">
         <v>Used Watermelon (pcs)</v>
       </c>
-      <c r="V3" t="str">
+      <c r="X3" t="str">
         <v>Used Mango</v>
       </c>
-      <c r="W3" t="str">
+      <c r="Y3" t="str">
         <v>Used Coco (Meat)</v>
       </c>
-      <c r="X3" t="str">
+      <c r="Z3" t="str">
         <v>Used Coco (Water)</v>
       </c>
-      <c r="Y3" t="str">
+      <c r="AA3" t="str">
         <v>Used Coco (Conden)</v>
       </c>
-      <c r="Z3" t="str">
+      <c r="AB3" t="str">
         <v>Used Coco (Raw)</v>
       </c>
-      <c r="AA3" t="str">
+      <c r="AC3" t="str">
         <v>Used Apple</v>
       </c>
-      <c r="AB3" t="str">
+      <c r="AD3" t="str">
         <v>Used Guava</v>
       </c>
-      <c r="AC3" t="str">
+      <c r="AE3" t="str">
         <v>Used Pineapple</v>
       </c>
-      <c r="AD3" t="str">
+      <c r="AF3" t="str">
         <v>Used Young Coco</v>
       </c>
-      <c r="AE3" t="str">
+      <c r="AG3" t="str">
         <v>Bottle Revenue (฿)</v>
       </c>
-      <c r="AF3" t="str">
+      <c r="AH3" t="str">
         <v>Source Note</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AF3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
B4 Sep: pineapple cups moved out of Apple, 29/09 mango, 30/09 volcano watermelon; fix pineapple/mangosteen fruit mapping (approved by Parn)
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B4_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B4_2026.xlsx
@@ -134,10 +134,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -169,10 +169,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1095,7 +1095,7 @@
         <v>0</v>
       </c>
       <c r="M9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -1104,7 +1104,7 @@
         <v>0</v>
       </c>
       <c r="P9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q9">
         <v>1</v>
@@ -1199,7 +1199,7 @@
         <v>0</v>
       </c>
       <c r="M10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -1208,7 +1208,7 @@
         <v>1</v>
       </c>
       <c r="P10">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q10">
         <v>4</v>
@@ -1303,7 +1303,7 @@
         <v>0</v>
       </c>
       <c r="M11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -1312,7 +1312,7 @@
         <v>3</v>
       </c>
       <c r="P11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q11">
         <v>7</v>
@@ -1401,13 +1401,13 @@
         <v>6</v>
       </c>
       <c r="K12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L12">
         <v>0</v>
       </c>
       <c r="M12">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N12">
         <v>0</v>
@@ -1416,7 +1416,7 @@
         <v>0</v>
       </c>
       <c r="P12">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q12">
         <v>8</v>
@@ -1502,13 +1502,13 @@
         <v>0</v>
       </c>
       <c r="J13">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="K13">
         <v>2</v>
       </c>
       <c r="L13">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M13">
         <v>1</v>

</xml_diff>